<commit_message>
docs(schema): 건조 성능 Output에 Tier 1(제품 KPI) 추가
Tier 2까지를 사이클까지로만 잡았던 것 수정 — Tier 1(건조성능 본체) 누적 포함.
- Product(Tier1) 9개 추가: SMER, drying_time, energy_consumption, energy_grade,
  MER, final_moisture, fabric_T_max, uniformity, total_condensate
- source=System: 드럼+과도해석 통합 산출(정상상태 단독 불가)
- 총 45개 (Product 9 + Component 17 + Cycle 19), core 23
- Tier 3(transient 곡선)만 미포함
</commit_message>
<xml_diff>
--- a/data/schema/HPWD_HX_PerformanceOutputs.xlsx
+++ b/data/schema/HPWD_HX_PerformanceOutputs.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL_DDL" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Performance_Outputs'!$A$1:$G$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Performance_Outputs'!$A$1:$G$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -54,7 +54,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -68,17 +68,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FECACA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E0F2FE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F1F5F9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -128,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -161,6 +171,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -529,11 +545,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
@@ -581,17 +597,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Product(Tier1)</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Q_total</t>
+          <t>SMER</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>System</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -606,29 +622,29 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>kg/kWh</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
-          <t>총 열교환량. 증발기=냉각량, 응축기=가열량. 사이클·건조 성능의 1차 재료</t>
+          <t>단위 소비전력당 제습량 = 누적 제습량/누적 소비전력. 건조 효율 최상위 지표</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Product(Tier1)</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Q_sensible</t>
+          <t>drying_time</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>System</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -636,36 +652,36 @@
           <t>float</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>min</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>현열 교환량(온도 변화분)</t>
+          <t>목표 수분율 도달까지 걸린 시간</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Product(Tier1)</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Q_latent</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Evap</t>
+          <t>energy_consumption</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>System</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -680,34 +696,34 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>kWh</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>잠열 교환량(제습분). 증발기 결로 시. 응축기는 0</t>
+          <t>1회 건조 사이클 총 소비 전력량</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Product(Tier1)</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>T_ref_out</t>
+          <t>energy_grade</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>System</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -717,29 +733,29 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>°C</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>냉매 출구 온도</t>
+          <t>에너지 효율 등급(IEC 61121 / 에너지라벨 기준)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Product(Tier1)</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>x_out</t>
+          <t>MER</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>System</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -754,29 +770,29 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>kg/h</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>냉매 출구 건도(quality)</t>
+          <t>시간당 평균 제습 속도</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Product(Tier1)</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>SH_out</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Evap</t>
+          <t>final_moisture</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>System</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -791,29 +807,29 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>%</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>증발기 출구 과열도. 압축기 흡입 보호·제어 타깃</t>
+          <t>건조 종료 시 직물 수분율(cupboard dry 등 목표 도달 여부)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Product(Tier1)</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>SC_out</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Cond</t>
+          <t>fabric_T_max</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>System</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -828,29 +844,29 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>°C</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>응축기 출구 과냉도. 충전량·EEV 거동 연계</t>
+          <t>건조 중 직물 최고 온도. 손상·구김 방지 제약</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Product(Tier1)</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>T_air_out</t>
+          <t>uniformity</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>System</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -858,1060 +874,1393 @@
           <t>float</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>Y</t>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>°C</t>
+          <t>%</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>공기 출구 온도. 응축기 출구=드럼 입구 온도로 건조 성능 직결</t>
+          <t>직물 위치별 수분 편차(건조 균일도)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Product(Tier1)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>total_condensate</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>사이클 누적 응축수량(총 제습량)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Q_total</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>총 열교환량. 증발기=냉각량, 응축기=가열량. 사이클·건조 성능의 1차 재료</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Q_sensible</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>현열 교환량(온도 변화분)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Q_latent</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Evap</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>잠열 교환량(제습분). 증발기 결로 시. 응축기는 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>T_ref_out</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>냉매 출구 온도</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>x_out</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>냉매 출구 건도(quality)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>SH_out</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Evap</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>증발기 출구 과열도. 압축기 흡입 보호·제어 타깃</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>SC_out</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Cond</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>응축기 출구 과냉도. 충전량·EEV 거동 연계</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>T_air_out</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>공기 출구 온도. 응축기 출구=드럼 입구 온도로 건조 성능 직결</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>RH_air_out</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>공기 출구 상대습도(절대습도 omega_out 병행)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>m_condensate</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>Evap</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>kg/s</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>응축수량(제습 속도). 증발기. MER·SMER의 직접 원천</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>dP_ref</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>Pa</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>냉매측 압력강하. 사이클 압력비·압축일 영향</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>dP_air</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>Pa</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>공기측 압력강하. 팬 운전점·풍량 결정 → 건조 성능 영향</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>M_holdup</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
         <is>
           <t>냉매 충전량(holdup). 시스템 charge balance 입력</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>UA_total</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>W/K</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>총 전열 컨덕턴스. 사이징·진단</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>eta_fin</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F25" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G25" s="7" t="inlineStr">
         <is>
           <t>핀 효율(진단)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>alpha_air</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>W/m²K</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G26" s="7" t="inlineStr">
         <is>
           <t>공기측 열전달계수(진단)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>alpha_ref</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>W/m²K</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="G27" s="7" t="inlineStr">
         <is>
           <t>냉매측 열전달계수(진단)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>COP</t>
         </is>
       </c>
-      <c r="C19" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="G28" s="7" t="inlineStr">
         <is>
           <t>성능계수 = Q_heating / W_total. 사이클 효율 핵심 지표</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>W_total</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G29" s="7" t="inlineStr">
         <is>
           <t>총 소비전력(압축기+팬). 에너지 소비·SMER 분모</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>W_comp</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F30" s="5" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="G30" s="7" t="inlineStr">
         <is>
           <t>압축기 소비전력. 전체 전력의 주성분</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>W_fan</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G31" s="7" t="inlineStr">
         <is>
           <t>팬 소비전력</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>T_e</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F32" s="5" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="G32" s="7" t="inlineStr">
         <is>
           <t>증발 온도. 제습 능력·착상 여부 결정</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>T_c</t>
         </is>
       </c>
-      <c r="C24" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="F33" s="5" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="G33" s="7" t="inlineStr">
         <is>
           <t>응축 온도. 드럼 가열 온도·압력 상한 연계</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>T_dis</t>
         </is>
       </c>
-      <c r="C25" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F34" s="5" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="G34" s="7" t="inlineStr">
         <is>
           <t>압축기 토출 온도. 보호 제약(상한 ~130°C, R290)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>P_e</t>
         </is>
       </c>
-      <c r="C26" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F35" s="5" t="inlineStr">
         <is>
           <t>bar</t>
         </is>
       </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="G35" s="7" t="inlineStr">
         <is>
           <t>증발 압력</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>P_c</t>
         </is>
       </c>
-      <c r="C27" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F36" s="5" t="inlineStr">
         <is>
           <t>bar</t>
         </is>
       </c>
-      <c r="G27" s="7" t="inlineStr">
+      <c r="G36" s="7" t="inlineStr">
         <is>
           <t>응축 압력. 설계압력 상한 제약(R290 ~25bar)</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>pressure_ratio</t>
         </is>
       </c>
-      <c r="C28" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="F37" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G37" s="7" t="inlineStr">
         <is>
           <t>압력비 P_c/P_e. 압축 효율 영향</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>m_dot_ref</t>
         </is>
       </c>
-      <c r="C29" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F38" s="5" t="inlineStr">
         <is>
           <t>kg/s</t>
         </is>
       </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="G38" s="7" t="inlineStr">
         <is>
           <t>냉매 순환유량. 사이클 용량 결정</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>SH_cycle</t>
         </is>
       </c>
-      <c r="C30" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="C39" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="F39" s="5" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="G39" s="7" t="inlineStr">
         <is>
           <t>사이클 과열도(제어 타깃)</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>SC_cycle</t>
         </is>
       </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F40" s="5" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="G40" s="7" t="inlineStr">
         <is>
           <t>사이클 과냉도(충전량 의존)</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>Q_heating</t>
         </is>
       </c>
-      <c r="C32" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="C41" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F32" s="5" t="inlineStr">
+      <c r="F41" s="5" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G32" s="7" t="inlineStr">
+      <c r="G41" s="7" t="inlineStr">
         <is>
           <t>응축기 가열량 = 드럼 입구 공기 가열. 건조 추진력</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>Q_cooling</t>
         </is>
       </c>
-      <c r="C33" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="C42" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="F42" s="5" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="G42" s="7" t="inlineStr">
         <is>
           <t>증발기 냉각량 = 제습 능력</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>T_air_drum_in</t>
         </is>
       </c>
-      <c r="C34" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="inlineStr">
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F34" s="5" t="inlineStr">
+      <c r="F43" s="5" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="G43" s="7" t="inlineStr">
         <is>
           <t>드럼 입구 공기 온도(응축기 출구). 건조 성능 직접 추진 변수</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>omega_drum_in</t>
         </is>
       </c>
-      <c r="C35" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
+      <c r="C44" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
+      <c r="F44" s="5" t="inlineStr">
         <is>
           <t>kg/kg</t>
         </is>
       </c>
-      <c r="G35" s="7" t="inlineStr">
+      <c r="G44" s="7" t="inlineStr">
         <is>
           <t>드럼 입구 공기 절대습도(증발기 제습 후)</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>charge_margin</t>
         </is>
       </c>
-      <c r="C36" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
+      <c r="C45" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
+      <c r="F45" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G36" s="7" t="inlineStr">
+      <c r="G45" s="7" t="inlineStr">
         <is>
           <t>충전량 적정성(과충전/부족 진단)</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>converged</t>
         </is>
       </c>
-      <c r="C37" s="11" t="inlineStr">
-        <is>
-          <t>Cycle</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
+      <c r="C46" s="13" t="inlineStr">
+        <is>
+          <t>Cycle</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
         <is>
           <t>bool</t>
         </is>
       </c>
-      <c r="E37" s="5" t="inlineStr">
+      <c r="E46" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
+      <c r="F46" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G37" s="7" t="inlineStr">
+      <c r="G46" s="7" t="inlineStr">
         <is>
           <t>사이클 연립 수렴 플래그</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G37"/>
+  <autoFilter ref="A1:G46"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1922,356 +2271,419 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A51"/>
+  <dimension ref="A1:A60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
-        <is>
-          <t>-- HPWD Studio · 건조 성능 Output 스키마 (Tier 2까지)</t>
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>-- HPWD Studio · 건조 성능 Output 스키마 (Tier 1 + Tier 2)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>-- Component = 증발기/응축기 HX 자체 출력 / Cycle = 사이클 정상상태(Tier 2).</t>
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>-- Product(Tier1)=제품/규격 건조성능 KPI / Cycle(Tier2)=사이클 정상상태 / Component=HX 자체 출력.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>-- Tier 1(SMER·건조시간 등 제품 KPI)과 Tier 3(transient 곡선)은 미포함.</t>
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>-- Tier 3(transient 곡선)은 미포함.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>-- source: Evap=증발기만, Cond=응축기만, Both=공통, Cycle=사이클 연립.</t>
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>-- source: Evap=증발기, Cond=응축기, Both=공통, Cycle=사이클 연립, System=드럼+과도해석 통합(정상상태 단독 산출 불가).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr"/>
+      <c r="A5" s="14" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>CREATE TABLE hx_performance_outputs (</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    output_name  VARCHAR(20)  PRIMARY KEY,</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    layer        VARCHAR(12)  NOT NULL CHECK (layer IN ('Component','Cycle')),</t>
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    layer        VARCHAR(16)  NOT NULL CHECK (layer IN ('Product(Tier1)','Component','Cycle')),</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    source       VARCHAR(8)   NOT NULL CHECK (source IN ('Evap','Cond','Both','Cycle')),</t>
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    source       VARCHAR(8)   NOT NULL CHECK (source IN ('Evap','Cond','Both','Cycle','System')),</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    dtype        VARCHAR(8)   NOT NULL CHECK (dtype IN ('float','int','bool')),</t>
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    dtype        VARCHAR(8)   NOT NULL CHECK (dtype IN ('float','int','bool','enum')),</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    is_core      BOOLEAN      NOT NULL DEFAULT FALSE,</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    unit         VARCHAR(8),</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    description  TEXT</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>);</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr"/>
+      <c r="A15" s="14" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>INSERT INTO hx_performance_outputs VALUES ('SMER','Product(Tier1)','System','float',TRUE,'kg/kWh','단위 소비전력당 제습량 = 누적 제습량/누적 소비전력. 건조 효율 최상위 지표');</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>INSERT INTO hx_performance_outputs VALUES ('drying_time','Product(Tier1)','System','float',TRUE,'min','목표 수분율 도달까지 걸린 시간');</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>INSERT INTO hx_performance_outputs VALUES ('energy_consumption','Product(Tier1)','System','float',TRUE,'kWh','1회 건조 사이클 총 소비 전력량');</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>INSERT INTO hx_performance_outputs VALUES ('energy_grade','Product(Tier1)','System','enum',TRUE,'-','에너지 효율 등급(IEC 61121 / 에너지라벨 기준)');</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>INSERT INTO hx_performance_outputs VALUES ('MER','Product(Tier1)','System','float',FALSE,'kg/h','시간당 평균 제습 속도');</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>INSERT INTO hx_performance_outputs VALUES ('final_moisture','Product(Tier1)','System','float',TRUE,'%','건조 종료 시 직물 수분율(cupboard dry 등 목표 도달 여부)');</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>INSERT INTO hx_performance_outputs VALUES ('fabric_T_max','Product(Tier1)','System','float',TRUE,'°C','건조 중 직물 최고 온도. 손상·구김 방지 제약');</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>INSERT INTO hx_performance_outputs VALUES ('uniformity','Product(Tier1)','System','float',FALSE,'%','직물 위치별 수분 편차(건조 균일도)');</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>INSERT INTO hx_performance_outputs VALUES ('total_condensate','Product(Tier1)','System','float',FALSE,'L','사이클 누적 응축수량(총 제습량)');</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('Q_total','Component','Both','float',TRUE,'W','총 열교환량. 증발기=냉각량, 응축기=가열량. 사이클·건조 성능의 1차 재료');</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('Q_sensible','Component','Both','float',FALSE,'W','현열 교환량(온도 변화분)');</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('Q_latent','Component','Evap','float',TRUE,'W','잠열 교환량(제습분). 증발기 결로 시. 응축기는 0');</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('T_ref_out','Component','Both','float',TRUE,'°C','냉매 출구 온도');</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="12" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('x_out','Component','Both','float',FALSE,'-','냉매 출구 건도(quality)');</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="12" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('SH_out','Component','Evap','float',TRUE,'K','증발기 출구 과열도. 압축기 흡입 보호·제어 타깃');</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="12" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('SC_out','Component','Cond','float',TRUE,'K','응축기 출구 과냉도. 충전량·EEV 거동 연계');</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="12" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('T_air_out','Component','Both','float',TRUE,'°C','공기 출구 온도. 응축기 출구=드럼 입구 온도로 건조 성능 직결');</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('RH_air_out','Component','Both','float',FALSE,'%','공기 출구 상대습도(절대습도 omega_out 병행)');</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="12" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('m_condensate','Component','Evap','float',TRUE,'kg/s','응축수량(제습 속도). 증발기. MER·SMER의 직접 원천');</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="12" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('dP_ref','Component','Both','float',FALSE,'Pa','냉매측 압력강하. 사이클 압력비·압축일 영향');</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="12" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('dP_air','Component','Both','float',TRUE,'Pa','공기측 압력강하. 팬 운전점·풍량 결정 → 건조 성능 영향');</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="12" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('M_holdup','Component','Both','float',FALSE,'kg','냉매 충전량(holdup). 시스템 charge balance 입력');</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="12" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('UA_total','Component','Both','float',FALSE,'W/K','총 전열 컨덕턴스. 사이징·진단');</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('eta_fin','Component','Both','float',FALSE,'-','핀 효율(진단)');</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="12" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('alpha_air','Component','Both','float',FALSE,'W/m²K','공기측 열전달계수(진단)');</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="12" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('alpha_ref','Component','Both','float',FALSE,'W/m²K','냉매측 열전달계수(진단)');</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="12" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('COP','Cycle','Cycle','float',TRUE,'-','성능계수 = Q_heating / W_total. 사이클 효율 핵심 지표');</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="12" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('W_total','Cycle','Cycle','float',TRUE,'W','총 소비전력(압축기+팬). 에너지 소비·SMER 분모');</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="12" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('W_comp','Cycle','Cycle','float',TRUE,'W','압축기 소비전력. 전체 전력의 주성분');</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="12" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('W_fan','Cycle','Cycle','float',FALSE,'W','팬 소비전력');</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="12" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('T_e','Cycle','Cycle','float',TRUE,'°C','증발 온도. 제습 능력·착상 여부 결정');</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="12" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('T_c','Cycle','Cycle','float',TRUE,'°C','응축 온도. 드럼 가열 온도·압력 상한 연계');</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="12" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('T_dis','Cycle','Cycle','float',TRUE,'°C','압축기 토출 온도. 보호 제약(상한 ~130°C, R290)');</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="12" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('P_e','Cycle','Cycle','float',FALSE,'bar','증발 압력');</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="12" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('P_c','Cycle','Cycle','float',FALSE,'bar','응축 압력. 설계압력 상한 제약(R290 ~25bar)');</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="12" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('pressure_ratio','Cycle','Cycle','float',FALSE,'-','압력비 P_c/P_e. 압축 효율 영향');</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="12" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('m_dot_ref','Cycle','Cycle','float',TRUE,'kg/s','냉매 순환유량. 사이클 용량 결정');</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="12" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('SH_cycle','Cycle','Cycle','float',FALSE,'K','사이클 과열도(제어 타깃)');</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="12" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('SC_cycle','Cycle','Cycle','float',FALSE,'K','사이클 과냉도(충전량 의존)');</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="12" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('Q_heating','Cycle','Cycle','float',TRUE,'W','응축기 가열량 = 드럼 입구 공기 가열. 건조 추진력');</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="12" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('Q_cooling','Cycle','Cycle','float',FALSE,'W','증발기 냉각량 = 제습 능력');</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="12" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('T_air_drum_in','Cycle','Cycle','float',TRUE,'°C','드럼 입구 공기 온도(응축기 출구). 건조 성능 직접 추진 변수');</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="12" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('omega_drum_in','Cycle','Cycle','float',FALSE,'kg/kg','드럼 입구 공기 절대습도(증발기 제습 후)');</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="12" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('charge_margin','Cycle','Cycle','float',FALSE,'-','충전량 적정성(과충전/부족 진단)');</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="12" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="14" t="inlineStr">
         <is>
           <t>INSERT INTO hx_performance_outputs VALUES ('converged','Cycle','Cycle','bool',FALSE,'-','사이클 연립 수렴 플래그');</t>
         </is>

</xml_diff>